<commit_message>
Workbook: candidate cards' powers as Action 1 / Action 2 / Action 3
The user: not a column per effect, but up to three actions per card.
Action 1 is always the draw (Draw N cards, blank if none); Actions 2
and 3 hold the rest as short phrases (Destroy up to N, Gain a story
costing N or less, Recover N, +N per kind played, Look at the top N,
Attack). Plain and candidate-theme influence keep their own columns,
as on the Stories sheet. No card uses Action 3 yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fourth-estate-cards.xlsx
+++ b/docs/fourth-estate-cards.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stories'!$A$1:$AC$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Elections'!$A$1:$AA$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Elections'!$A$1:$U$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Newspapers'!$A$1:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -642,28 +642,28 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>the power when played: Influence (plain); Candidate-theme influence (his theme); Draw; Destroy (up to N cards from hand or discard);</t>
+          <t>when played: Influence (plain) = plain influence; Candidate-theme influence = influence of his theme;</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Draw per destroyed (1 = draw a card for each); Gain (cost up to) a story from the exchange; Recover (cards from discard to hand);</t>
+          <t>Action 1 = the draw (Draw N cards; blank if none); Action 2 and Action 3 = its other actions: Destroy up to N cards (draw 1 for each),</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Per kind played (+N per different kind of card played this turn); Look at top (look at the top N of the main deck, keep 1);</t>
+          <t>Gain a story costing N or less, Recover N cards from discard, +N influence per kind of card played, Look at the top N (keep 1),</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Stays in play (+N each turn; none now); Attack (discard or scandal, every rival); Power = the card's text.</t>
+          <t>Attack (each rival discards a card / gains a Scandal); Power = the card's full text.</t>
         </is>
       </c>
     </row>
@@ -11623,7 +11623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA35"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11639,20 +11639,14 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="9" customWidth="1" min="22" max="22"/>
-    <col width="55" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="45" customWidth="1" min="25" max="25"/>
-    <col width="10" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="45" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -11723,70 +11717,40 @@
       </c>
       <c r="N1" s="4" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Action 1</t>
         </is>
       </c>
       <c r="O1" s="4" t="inlineStr">
         <is>
-          <t>Destroy</t>
+          <t>Action 2</t>
         </is>
       </c>
       <c r="P1" s="4" t="inlineStr">
         <is>
-          <t>Draw per destroyed</t>
+          <t>Action 3</t>
         </is>
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
-          <t>Gain (cost up to)</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="R1" s="4" t="inlineStr">
         <is>
-          <t>Recover</t>
+          <t>fa_name</t>
         </is>
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
-          <t>Per kind played</t>
+          <t>First Appearance</t>
         </is>
       </c>
       <c r="T1" s="4" t="inlineStr">
         <is>
-          <t>Look at top</t>
+          <t>fa_kind</t>
         </is>
       </c>
       <c r="U1" s="4" t="inlineStr">
-        <is>
-          <t>Stays in play</t>
-        </is>
-      </c>
-      <c r="V1" s="4" t="inlineStr">
-        <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="W1" s="4" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="X1" s="4" t="inlineStr">
-        <is>
-          <t>fa_name</t>
-        </is>
-      </c>
-      <c r="Y1" s="4" t="inlineStr">
-        <is>
-          <t>First Appearance</t>
-        </is>
-      </c>
-      <c r="Z1" s="4" t="inlineStr">
-        <is>
-          <t>fa_kind</t>
-        </is>
-      </c>
-      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>First Appearance: how many</t>
         </is>
@@ -11846,40 +11810,22 @@
       <c r="M2" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>+2 influence, draw a card.</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="5" t="n"/>
       <c r="U2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" s="5" t="n"/>
-      <c r="W2" s="6" t="inlineStr">
-        <is>
-          <t>+2 influence, draw a card.</t>
-        </is>
-      </c>
-      <c r="X2" s="6" t="n"/>
-      <c r="Y2" s="6" t="n"/>
-      <c r="Z2" s="5" t="n"/>
-      <c r="AA2" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11933,40 +11879,22 @@
       <c r="M3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Draw 2 cards</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
+      <c r="Q3" s="6" t="inlineStr">
+        <is>
+          <t>Draw 2 cards.</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="n"/>
+      <c r="S3" s="6" t="n"/>
+      <c r="T3" s="5" t="n"/>
       <c r="U3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="5" t="n"/>
-      <c r="W3" s="6" t="inlineStr">
-        <is>
-          <t>Draw 2 cards.</t>
-        </is>
-      </c>
-      <c r="X3" s="6" t="n"/>
-      <c r="Y3" s="6" t="n"/>
-      <c r="Z3" s="5" t="n"/>
-      <c r="AA3" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12020,56 +11948,34 @@
       <c r="M4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="7" t="n">
-        <v>0</v>
+      <c r="N4" s="8" t="n"/>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>Attack: each rival discards a card</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="n"/>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>+2 influence. Attack: each rival paper discards a card at random.</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>The Sedition Act</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards a card at random.</t>
+        </is>
+      </c>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="7" t="inlineStr">
-        <is>
-          <t>discard</t>
-        </is>
-      </c>
-      <c r="W4" s="8" t="inlineStr">
-        <is>
-          <t>+2 influence. Attack: each rival paper discards a card at random.</t>
-        </is>
-      </c>
-      <c r="X4" s="8" t="inlineStr">
-        <is>
-          <t>The Sedition Act</t>
-        </is>
-      </c>
-      <c r="Y4" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards a card at random.</t>
-        </is>
-      </c>
-      <c r="Z4" s="7" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA4" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12127,52 +12033,38 @@
       <c r="M5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N5" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="7" t="n">
-        <v>0</v>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Draw 2 cards</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>Destroy up to 1 card</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="n"/>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>+2 influence, draw 2 cards, then you may destroy a card in your hand or discard pile.</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>The Sedition Act</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards a card at random.</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="7" t="n"/>
-      <c r="W5" s="8" t="inlineStr">
-        <is>
-          <t>+2 influence, draw 2 cards, then you may destroy a card in your hand or discard pile.</t>
-        </is>
-      </c>
-      <c r="X5" s="8" t="inlineStr">
-        <is>
-          <t>The Sedition Act</t>
-        </is>
-      </c>
-      <c r="Y5" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards a card at random.</t>
-        </is>
-      </c>
-      <c r="Z5" s="7" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA5" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12230,52 +12122,34 @@
       <c r="M6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="R6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="5" t="n">
-        <v>0</v>
+      <c r="N6" s="6" t="n"/>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>Gain a story costing 4 or less</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>+2 influence. Gain a story costing 4 or less from the exchange.</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>The Twelfth Amendment</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>Each paper draws a card.</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
       </c>
       <c r="U6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="6" t="inlineStr">
-        <is>
-          <t>+2 influence. Gain a story costing 4 or less from the exchange.</t>
-        </is>
-      </c>
-      <c r="X6" s="6" t="inlineStr">
-        <is>
-          <t>The Twelfth Amendment</t>
-        </is>
-      </c>
-      <c r="Y6" s="6" t="inlineStr">
-        <is>
-          <t>Each paper draws a card.</t>
-        </is>
-      </c>
-      <c r="Z6" s="5" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="AA6" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12329,52 +12203,34 @@
       <c r="M7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="5" t="n">
-        <v>0</v>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>Destroy up to 1 card</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="n"/>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>+3 influence, then you may destroy a card in your hand or discard pile.</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>The Twelfth Amendment</t>
+        </is>
+      </c>
+      <c r="S7" s="6" t="inlineStr">
+        <is>
+          <t>Each paper draws a card.</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
       </c>
       <c r="U7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>+3 influence, then you may destroy a card in your hand or discard pile.</t>
-        </is>
-      </c>
-      <c r="X7" s="6" t="inlineStr">
-        <is>
-          <t>The Twelfth Amendment</t>
-        </is>
-      </c>
-      <c r="Y7" s="6" t="inlineStr">
-        <is>
-          <t>Each paper draws a card.</t>
-        </is>
-      </c>
-      <c r="Z7" s="5" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="AA7" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12432,52 +12288,30 @@
       <c r="M8" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="7" t="n">
-        <v>0</v>
+      <c r="N8" s="8" t="n"/>
+      <c r="O8" s="8" t="n"/>
+      <c r="P8" s="8" t="n"/>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>+4 influence.</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>The Embargo</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
+          <t>Each paper discards the most expensive card in its hand.</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>discard_dearest</t>
+        </is>
       </c>
       <c r="U8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="8" t="inlineStr">
-        <is>
-          <t>+4 influence.</t>
-        </is>
-      </c>
-      <c r="X8" s="8" t="inlineStr">
-        <is>
-          <t>The Embargo</t>
-        </is>
-      </c>
-      <c r="Y8" s="8" t="inlineStr">
-        <is>
-          <t>Each paper discards the most expensive card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z8" s="7" t="inlineStr">
-        <is>
-          <t>discard_dearest</t>
-        </is>
-      </c>
-      <c r="AA8" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12531,52 +12365,34 @@
       <c r="M9" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="R9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="7" t="n">
-        <v>0</v>
+      <c r="N9" s="8" t="n"/>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>Gain a story costing 5 or less</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="n"/>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>Gain a story costing 5 or less from the exchange.</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>The Embargo</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>Each paper discards the most expensive card in its hand.</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>discard_dearest</t>
+        </is>
       </c>
       <c r="U9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="8" t="inlineStr">
-        <is>
-          <t>Gain a story costing 5 or less from the exchange.</t>
-        </is>
-      </c>
-      <c r="X9" s="8" t="inlineStr">
-        <is>
-          <t>The Embargo</t>
-        </is>
-      </c>
-      <c r="Y9" s="8" t="inlineStr">
-        <is>
-          <t>Each paper discards the most expensive card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z9" s="7" t="inlineStr">
-        <is>
-          <t>discard_dearest</t>
-        </is>
-      </c>
-      <c r="AA9" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12634,52 +12450,34 @@
       <c r="M10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="5" t="n">
-        <v>0</v>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>+1 influence per kind of card played</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="n"/>
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>+1 influence for each different kind of card you play this turn.</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>Impressment</t>
+        </is>
+      </c>
+      <c r="S10" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="6" t="inlineStr">
-        <is>
-          <t>+1 influence for each different kind of card you play this turn.</t>
-        </is>
-      </c>
-      <c r="X10" s="6" t="inlineStr">
-        <is>
-          <t>Impressment</t>
-        </is>
-      </c>
-      <c r="Y10" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z10" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA10" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12733,52 +12531,34 @@
       <c r="M11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="5" t="n">
-        <v>0</v>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>Draw 2 cards</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="6" t="inlineStr">
+        <is>
+          <t>+2 influence, draw 2 cards.</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>Impressment</t>
+        </is>
+      </c>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T11" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="6" t="inlineStr">
-        <is>
-          <t>+2 influence, draw 2 cards.</t>
-        </is>
-      </c>
-      <c r="X11" s="6" t="inlineStr">
-        <is>
-          <t>Impressment</t>
-        </is>
-      </c>
-      <c r="Y11" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z11" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA11" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12836,52 +12616,34 @@
       <c r="M12" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N12" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="O12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="7" t="n">
-        <v>0</v>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>Draw 3 cards</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="n"/>
+      <c r="P12" s="8" t="n"/>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>Draw 3 cards.</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>Good Feelings</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>Each paper destroys a Scandal in its hand or discard pile.</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>unscandal</t>
+        </is>
       </c>
       <c r="U12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="8" t="inlineStr">
-        <is>
-          <t>Draw 3 cards.</t>
-        </is>
-      </c>
-      <c r="X12" s="8" t="inlineStr">
-        <is>
-          <t>Good Feelings</t>
-        </is>
-      </c>
-      <c r="Y12" s="8" t="inlineStr">
-        <is>
-          <t>Each paper destroys a Scandal in its hand or discard pile.</t>
-        </is>
-      </c>
-      <c r="Z12" s="7" t="inlineStr">
-        <is>
-          <t>unscandal</t>
-        </is>
-      </c>
-      <c r="AA12" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12935,52 +12697,34 @@
       <c r="M13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="7" t="n">
-        <v>0</v>
+      <c r="N13" s="8" t="n"/>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>Recover 1 card from discard</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>+2 influence. Put a card from your discard pile into your hand.</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>Good Feelings</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>Each paper destroys a Scandal in its hand or discard pile.</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>unscandal</t>
+        </is>
       </c>
       <c r="U13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="8" t="inlineStr">
-        <is>
-          <t>+2 influence. Put a card from your discard pile into your hand.</t>
-        </is>
-      </c>
-      <c r="X13" s="8" t="inlineStr">
-        <is>
-          <t>Good Feelings</t>
-        </is>
-      </c>
-      <c r="Y13" s="8" t="inlineStr">
-        <is>
-          <t>Each paper destroys a Scandal in its hand or discard pile.</t>
-        </is>
-      </c>
-      <c r="Z13" s="7" t="inlineStr">
-        <is>
-          <t>unscandal</t>
-        </is>
-      </c>
-      <c r="AA13" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13034,52 +12778,34 @@
       <c r="M14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="5" t="n">
-        <v>3</v>
+      <c r="N14" s="6" t="n"/>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>Look at the top 3, keep 1</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="6" t="inlineStr">
+        <is>
+          <t>+1 influence. Look at the top 3 stories of the main deck; put one into your hand, the rest on the bottom.</t>
+        </is>
+      </c>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>A Fire Bell in the Night</t>
+        </is>
+      </c>
+      <c r="S14" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards a card at random.</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="6" t="inlineStr">
-        <is>
-          <t>+1 influence. Look at the top 3 stories of the main deck; put one into your hand, the rest on the bottom.</t>
-        </is>
-      </c>
-      <c r="X14" s="6" t="inlineStr">
-        <is>
-          <t>A Fire Bell in the Night</t>
-        </is>
-      </c>
-      <c r="Y14" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards a card at random.</t>
-        </is>
-      </c>
-      <c r="Z14" s="5" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA14" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13137,52 +12863,34 @@
       <c r="M15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="5" t="n">
-        <v>0</v>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>Destroy up to 2 cards, draw 1 for each</t>
+        </is>
+      </c>
+      <c r="P15" s="6" t="n"/>
+      <c r="Q15" s="6" t="inlineStr">
+        <is>
+          <t>Destroy up to 2 cards in your hand or discard pile; draw a card for each.</t>
+        </is>
+      </c>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>A Fire Bell in the Night</t>
+        </is>
+      </c>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards a card at random.</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" s="5" t="n"/>
-      <c r="W15" s="6" t="inlineStr">
-        <is>
-          <t>Destroy up to 2 cards in your hand or discard pile; draw a card for each.</t>
-        </is>
-      </c>
-      <c r="X15" s="6" t="inlineStr">
-        <is>
-          <t>A Fire Bell in the Night</t>
-        </is>
-      </c>
-      <c r="Y15" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards a card at random.</t>
-        </is>
-      </c>
-      <c r="Z15" s="5" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA15" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13240,52 +12948,34 @@
       <c r="M16" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="S16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="7" t="n">
-        <v>0</v>
+      <c r="N16" s="8" t="n"/>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>Recover 2 cards from discard</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="n"/>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>Put up to 2 cards from your discard pile into your hand.</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>The Corrupt Bargain</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" s="7" t="n"/>
-      <c r="W16" s="8" t="inlineStr">
-        <is>
-          <t>Put up to 2 cards from your discard pile into your hand.</t>
-        </is>
-      </c>
-      <c r="X16" s="8" t="inlineStr">
-        <is>
-          <t>The Corrupt Bargain</t>
-        </is>
-      </c>
-      <c r="Y16" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z16" s="7" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA16" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13339,52 +13029,34 @@
       <c r="M17" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N17" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" s="7" t="n">
-        <v>0</v>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="n"/>
+      <c r="P17" s="8" t="n"/>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>+4 influence, draw a card.</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>The Corrupt Bargain</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" s="7" t="n"/>
-      <c r="W17" s="8" t="inlineStr">
-        <is>
-          <t>+4 influence, draw a card.</t>
-        </is>
-      </c>
-      <c r="X17" s="8" t="inlineStr">
-        <is>
-          <t>The Corrupt Bargain</t>
-        </is>
-      </c>
-      <c r="Y17" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z17" s="7" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA17" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13438,52 +13110,38 @@
       <c r="M18" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="R18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="5" t="n">
-        <v>0</v>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>Gain a story costing 5 or less</t>
+        </is>
+      </c>
+      <c r="P18" s="6" t="n"/>
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>Gain a story costing 5 or less from the exchange. Draw a card.</t>
+        </is>
+      </c>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>Mudslinging</t>
+        </is>
+      </c>
+      <c r="S18" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" s="5" t="n"/>
-      <c r="W18" s="6" t="inlineStr">
-        <is>
-          <t>Gain a story costing 5 or less from the exchange. Draw a card.</t>
-        </is>
-      </c>
-      <c r="X18" s="6" t="inlineStr">
-        <is>
-          <t>Mudslinging</t>
-        </is>
-      </c>
-      <c r="Y18" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z18" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA18" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13541,52 +13199,34 @@
       <c r="M19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="5" t="n">
-        <v>0</v>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
+      <c r="Q19" s="6" t="inlineStr">
+        <is>
+          <t>+3 influence, draw a card.</t>
+        </is>
+      </c>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>Mudslinging</t>
+        </is>
+      </c>
+      <c r="S19" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="5" t="n"/>
-      <c r="W19" s="6" t="inlineStr">
-        <is>
-          <t>+3 influence, draw a card.</t>
-        </is>
-      </c>
-      <c r="X19" s="6" t="inlineStr">
-        <is>
-          <t>Mudslinging</t>
-        </is>
-      </c>
-      <c r="Y19" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z19" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA19" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13640,52 +13280,34 @@
       <c r="M20" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="R20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="7" t="n">
-        <v>0</v>
+      <c r="N20" s="8" t="n"/>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>Gain a story costing 4 or less</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="n"/>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>+3 influence. Gain a story costing 4 or less from the exchange.</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t>The Veto</t>
+        </is>
+      </c>
+      <c r="S20" s="8" t="inlineStr">
+        <is>
+          <t>The exchange is swept and dealt afresh.</t>
+        </is>
+      </c>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>sweep</t>
+        </is>
       </c>
       <c r="U20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="8" t="inlineStr">
-        <is>
-          <t>+3 influence. Gain a story costing 4 or less from the exchange.</t>
-        </is>
-      </c>
-      <c r="X20" s="8" t="inlineStr">
-        <is>
-          <t>The Veto</t>
-        </is>
-      </c>
-      <c r="Y20" s="8" t="inlineStr">
-        <is>
-          <t>The exchange is swept and dealt afresh.</t>
-        </is>
-      </c>
-      <c r="Z20" s="7" t="inlineStr">
-        <is>
-          <t>sweep</t>
-        </is>
-      </c>
-      <c r="AA20" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13743,52 +13365,38 @@
       <c r="M21" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="R21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" s="7" t="n">
-        <v>0</v>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr">
+        <is>
+          <t>Gain a story costing 6 or less</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="n"/>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>Gain a story costing 6 or less from the exchange. Draw a card.</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>The Veto</t>
+        </is>
+      </c>
+      <c r="S21" s="8" t="inlineStr">
+        <is>
+          <t>The exchange is swept and dealt afresh.</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>sweep</t>
+        </is>
       </c>
       <c r="U21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V21" s="7" t="n"/>
-      <c r="W21" s="8" t="inlineStr">
-        <is>
-          <t>Gain a story costing 6 or less from the exchange. Draw a card.</t>
-        </is>
-      </c>
-      <c r="X21" s="8" t="inlineStr">
-        <is>
-          <t>The Veto</t>
-        </is>
-      </c>
-      <c r="Y21" s="8" t="inlineStr">
-        <is>
-          <t>The exchange is swept and dealt afresh.</t>
-        </is>
-      </c>
-      <c r="Z21" s="7" t="inlineStr">
-        <is>
-          <t>sweep</t>
-        </is>
-      </c>
-      <c r="AA21" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -13842,52 +13450,34 @@
       <c r="M22" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="T22" s="5" t="n">
-        <v>0</v>
+      <c r="N22" s="6" t="n"/>
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>+1 influence per kind of card played</t>
+        </is>
+      </c>
+      <c r="P22" s="6" t="n"/>
+      <c r="Q22" s="6" t="inlineStr">
+        <is>
+          <t>+2 influence, and +1 for each different kind of card you play this turn.</t>
+        </is>
+      </c>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>The Panic of 1837</t>
+        </is>
+      </c>
+      <c r="S22" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" s="5" t="n"/>
-      <c r="W22" s="6" t="inlineStr">
-        <is>
-          <t>+2 influence, and +1 for each different kind of card you play this turn.</t>
-        </is>
-      </c>
-      <c r="X22" s="6" t="inlineStr">
-        <is>
-          <t>The Panic of 1837</t>
-        </is>
-      </c>
-      <c r="Y22" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
-        </is>
-      </c>
-      <c r="Z22" s="5" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA22" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -13945,52 +13535,34 @@
       <c r="M23" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="N23" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" s="5" t="n">
-        <v>0</v>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>Draw 2 cards</t>
+        </is>
+      </c>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>+3 influence, draw 2 cards.</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>The Panic of 1837</t>
+        </is>
+      </c>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" s="5" t="n"/>
-      <c r="W23" s="6" t="inlineStr">
-        <is>
-          <t>+3 influence, draw 2 cards.</t>
-        </is>
-      </c>
-      <c r="X23" s="6" t="inlineStr">
-        <is>
-          <t>The Panic of 1837</t>
-        </is>
-      </c>
-      <c r="Y23" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
-        </is>
-      </c>
-      <c r="Z23" s="5" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA23" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14048,52 +13620,30 @@
       <c r="M24" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="7" t="n">
-        <v>0</v>
+      <c r="N24" s="8" t="n"/>
+      <c r="O24" s="8" t="n"/>
+      <c r="P24" s="8" t="n"/>
+      <c r="Q24" s="8" t="inlineStr">
+        <is>
+          <t>+4 influence.</t>
+        </is>
+      </c>
+      <c r="R24" s="8" t="inlineStr">
+        <is>
+          <t>Tippecanoe and Tyler Too</t>
+        </is>
+      </c>
+      <c r="S24" s="8" t="inlineStr">
+        <is>
+          <t>Each paper draws a card.</t>
+        </is>
+      </c>
+      <c r="T24" s="7" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
       </c>
       <c r="U24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" s="7" t="n"/>
-      <c r="W24" s="8" t="inlineStr">
-        <is>
-          <t>+4 influence.</t>
-        </is>
-      </c>
-      <c r="X24" s="8" t="inlineStr">
-        <is>
-          <t>Tippecanoe and Tyler Too</t>
-        </is>
-      </c>
-      <c r="Y24" s="8" t="inlineStr">
-        <is>
-          <t>Each paper draws a card.</t>
-        </is>
-      </c>
-      <c r="Z24" s="7" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="AA24" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14147,52 +13697,34 @@
       <c r="M25" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="N25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="P25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" s="7" t="n">
-        <v>0</v>
+      <c r="N25" s="8" t="n"/>
+      <c r="O25" s="8" t="inlineStr">
+        <is>
+          <t>Destroy up to 2 cards, draw 1 for each</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="n"/>
+      <c r="Q25" s="8" t="inlineStr">
+        <is>
+          <t>+2 influence. Destroy up to 2 cards in your hand or discard pile; draw a card for each.</t>
+        </is>
+      </c>
+      <c r="R25" s="8" t="inlineStr">
+        <is>
+          <t>Tippecanoe and Tyler Too</t>
+        </is>
+      </c>
+      <c r="S25" s="8" t="inlineStr">
+        <is>
+          <t>Each paper draws a card.</t>
+        </is>
+      </c>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
       </c>
       <c r="U25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V25" s="7" t="n"/>
-      <c r="W25" s="8" t="inlineStr">
-        <is>
-          <t>+2 influence. Destroy up to 2 cards in your hand or discard pile; draw a card for each.</t>
-        </is>
-      </c>
-      <c r="X25" s="8" t="inlineStr">
-        <is>
-          <t>Tippecanoe and Tyler Too</t>
-        </is>
-      </c>
-      <c r="Y25" s="8" t="inlineStr">
-        <is>
-          <t>Each paper draws a card.</t>
-        </is>
-      </c>
-      <c r="Z25" s="7" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="AA25" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14246,52 +13778,34 @@
       <c r="M26" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="S26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="5" t="n">
-        <v>0</v>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>Recover 1 card from discard</t>
+        </is>
+      </c>
+      <c r="P26" s="6" t="n"/>
+      <c r="Q26" s="6" t="inlineStr">
+        <is>
+          <t>+3 influence. Put a card from your discard pile into your hand.</t>
+        </is>
+      </c>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>Fifty-four Forty</t>
+        </is>
+      </c>
+      <c r="S26" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the fewest offices draws 2 cards.</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>draw_fewest</t>
+        </is>
       </c>
       <c r="U26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" s="5" t="n"/>
-      <c r="W26" s="6" t="inlineStr">
-        <is>
-          <t>+3 influence. Put a card from your discard pile into your hand.</t>
-        </is>
-      </c>
-      <c r="X26" s="6" t="inlineStr">
-        <is>
-          <t>Fifty-four Forty</t>
-        </is>
-      </c>
-      <c r="Y26" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the fewest offices draws 2 cards.</t>
-        </is>
-      </c>
-      <c r="Z26" s="5" t="inlineStr">
-        <is>
-          <t>draw_fewest</t>
-        </is>
-      </c>
-      <c r="AA26" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14349,52 +13863,34 @@
       <c r="M27" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="5" t="n">
-        <v>3</v>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="6" t="inlineStr">
+        <is>
+          <t>Look at the top 3, keep 1</t>
+        </is>
+      </c>
+      <c r="P27" s="6" t="n"/>
+      <c r="Q27" s="6" t="inlineStr">
+        <is>
+          <t>+2 influence. Look at the top 3 stories of the main deck; put one into your hand, the rest on the bottom.</t>
+        </is>
+      </c>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>Fifty-four Forty</t>
+        </is>
+      </c>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the fewest offices draws 2 cards.</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>draw_fewest</t>
+        </is>
       </c>
       <c r="U27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" s="5" t="n"/>
-      <c r="W27" s="6" t="inlineStr">
-        <is>
-          <t>+2 influence. Look at the top 3 stories of the main deck; put one into your hand, the rest on the bottom.</t>
-        </is>
-      </c>
-      <c r="X27" s="6" t="inlineStr">
-        <is>
-          <t>Fifty-four Forty</t>
-        </is>
-      </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the fewest offices draws 2 cards.</t>
-        </is>
-      </c>
-      <c r="Z27" s="5" t="inlineStr">
-        <is>
-          <t>draw_fewest</t>
-        </is>
-      </c>
-      <c r="AA27" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14452,56 +13948,34 @@
       <c r="M28" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="N28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="7" t="n">
-        <v>0</v>
+      <c r="N28" s="8" t="n"/>
+      <c r="O28" s="8" t="inlineStr">
+        <is>
+          <t>Attack: each rival discards a card</t>
+        </is>
+      </c>
+      <c r="P28" s="8" t="n"/>
+      <c r="Q28" s="8" t="inlineStr">
+        <is>
+          <t>+4 influence. Attack: each rival paper discards a card at random.</t>
+        </is>
+      </c>
+      <c r="R28" s="8" t="inlineStr">
+        <is>
+          <t>The Wilmot Proviso</t>
+        </is>
+      </c>
+      <c r="S28" s="8" t="inlineStr">
+        <is>
+          <t>Each paper destroys the cheapest card in its hand.</t>
+        </is>
+      </c>
+      <c r="T28" s="7" t="inlineStr">
+        <is>
+          <t>destroy_cheapest</t>
+        </is>
       </c>
       <c r="U28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V28" s="7" t="inlineStr">
-        <is>
-          <t>discard</t>
-        </is>
-      </c>
-      <c r="W28" s="8" t="inlineStr">
-        <is>
-          <t>+4 influence. Attack: each rival paper discards a card at random.</t>
-        </is>
-      </c>
-      <c r="X28" s="8" t="inlineStr">
-        <is>
-          <t>The Wilmot Proviso</t>
-        </is>
-      </c>
-      <c r="Y28" s="8" t="inlineStr">
-        <is>
-          <t>Each paper destroys the cheapest card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z28" s="7" t="inlineStr">
-        <is>
-          <t>destroy_cheapest</t>
-        </is>
-      </c>
-      <c r="AA28" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14555,52 +14029,38 @@
       <c r="M29" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="N29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="T29" s="7" t="n">
-        <v>0</v>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="inlineStr">
+        <is>
+          <t>+1 influence per kind of card played</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="n"/>
+      <c r="Q29" s="8" t="inlineStr">
+        <is>
+          <t>+1 influence for each different kind of card you play this turn. Draw a card.</t>
+        </is>
+      </c>
+      <c r="R29" s="8" t="inlineStr">
+        <is>
+          <t>The Wilmot Proviso</t>
+        </is>
+      </c>
+      <c r="S29" s="8" t="inlineStr">
+        <is>
+          <t>Each paper destroys the cheapest card in its hand.</t>
+        </is>
+      </c>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>destroy_cheapest</t>
+        </is>
       </c>
       <c r="U29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V29" s="7" t="n"/>
-      <c r="W29" s="8" t="inlineStr">
-        <is>
-          <t>+1 influence for each different kind of card you play this turn. Draw a card.</t>
-        </is>
-      </c>
-      <c r="X29" s="8" t="inlineStr">
-        <is>
-          <t>The Wilmot Proviso</t>
-        </is>
-      </c>
-      <c r="Y29" s="8" t="inlineStr">
-        <is>
-          <t>Each paper destroys the cheapest card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z29" s="7" t="inlineStr">
-        <is>
-          <t>destroy_cheapest</t>
-        </is>
-      </c>
-      <c r="AA29" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14654,52 +14114,34 @@
       <c r="M30" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" s="5" t="n">
-        <v>0</v>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>Draw 1 card</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="n"/>
+      <c r="P30" s="6" t="n"/>
+      <c r="Q30" s="6" t="inlineStr">
+        <is>
+          <t>+5 influence, draw a card.</t>
+        </is>
+      </c>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>The Fugitive Slave Act</t>
+        </is>
+      </c>
+      <c r="S30" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V30" s="5" t="n"/>
-      <c r="W30" s="6" t="inlineStr">
-        <is>
-          <t>+5 influence, draw a card.</t>
-        </is>
-      </c>
-      <c r="X30" s="6" t="inlineStr">
-        <is>
-          <t>The Fugitive Slave Act</t>
-        </is>
-      </c>
-      <c r="Y30" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z30" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA30" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14757,52 +14199,34 @@
       <c r="M31" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="P31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" s="5" t="n">
-        <v>0</v>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="6" t="inlineStr">
+        <is>
+          <t>Destroy up to 3 cards, draw 1 for each</t>
+        </is>
+      </c>
+      <c r="P31" s="6" t="n"/>
+      <c r="Q31" s="6" t="inlineStr">
+        <is>
+          <t>Destroy up to 3 cards in your hand or discard pile; draw a card for each.</t>
+        </is>
+      </c>
+      <c r="R31" s="6" t="inlineStr">
+        <is>
+          <t>The Fugitive Slave Act</t>
+        </is>
+      </c>
+      <c r="S31" s="6" t="inlineStr">
+        <is>
+          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>scandal_leader</t>
+        </is>
       </c>
       <c r="U31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" s="5" t="n"/>
-      <c r="W31" s="6" t="inlineStr">
-        <is>
-          <t>Destroy up to 3 cards in your hand or discard pile; draw a card for each.</t>
-        </is>
-      </c>
-      <c r="X31" s="6" t="inlineStr">
-        <is>
-          <t>The Fugitive Slave Act</t>
-        </is>
-      </c>
-      <c r="Y31" s="6" t="inlineStr">
-        <is>
-          <t>The paper (or papers) with the most prestige gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="Z31" s="5" t="inlineStr">
-        <is>
-          <t>scandal_leader</t>
-        </is>
-      </c>
-      <c r="AA31" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -14856,52 +14280,38 @@
       <c r="M32" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="N32" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="O32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" s="7" t="n">
-        <v>0</v>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
+          <t>Draw 2 cards</t>
+        </is>
+      </c>
+      <c r="O32" s="8" t="inlineStr">
+        <is>
+          <t>Destroy up to 1 card</t>
+        </is>
+      </c>
+      <c r="P32" s="8" t="n"/>
+      <c r="Q32" s="8" t="inlineStr">
+        <is>
+          <t>+3 influence, draw 2 cards, then you may destroy a card in your hand or discard pile.</t>
+        </is>
+      </c>
+      <c r="R32" s="8" t="inlineStr">
+        <is>
+          <t>Bleeding Kansas</t>
+        </is>
+      </c>
+      <c r="S32" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
+        </is>
+      </c>
+      <c r="T32" s="7" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V32" s="7" t="n"/>
-      <c r="W32" s="8" t="inlineStr">
-        <is>
-          <t>+3 influence, draw 2 cards, then you may destroy a card in your hand or discard pile.</t>
-        </is>
-      </c>
-      <c r="X32" s="8" t="inlineStr">
-        <is>
-          <t>Bleeding Kansas</t>
-        </is>
-      </c>
-      <c r="Y32" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
-        </is>
-      </c>
-      <c r="Z32" s="7" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA32" s="7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14959,56 +14369,34 @@
       <c r="M33" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="N33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" s="7" t="n">
-        <v>0</v>
+      <c r="N33" s="8" t="n"/>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>Attack: each rival gains a Scandal</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="n"/>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>+5 influence. Attack: each rival paper gains a Scandal.</t>
+        </is>
+      </c>
+      <c r="R33" s="8" t="inlineStr">
+        <is>
+          <t>Bleeding Kansas</t>
+        </is>
+      </c>
+      <c r="S33" s="8" t="inlineStr">
+        <is>
+          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
+        </is>
+      </c>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>discard_leader</t>
+        </is>
       </c>
       <c r="U33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" s="7" t="inlineStr">
-        <is>
-          <t>scandal</t>
-        </is>
-      </c>
-      <c r="W33" s="8" t="inlineStr">
-        <is>
-          <t>+5 influence. Attack: each rival paper gains a Scandal.</t>
-        </is>
-      </c>
-      <c r="X33" s="8" t="inlineStr">
-        <is>
-          <t>Bleeding Kansas</t>
-        </is>
-      </c>
-      <c r="Y33" s="8" t="inlineStr">
-        <is>
-          <t>The paper (or papers) holding the most offices discards 2 cards at random.</t>
-        </is>
-      </c>
-      <c r="Z33" s="7" t="inlineStr">
-        <is>
-          <t>discard_leader</t>
-        </is>
-      </c>
-      <c r="AA33" s="7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -15066,52 +14454,30 @@
       <c r="M34" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" s="5" t="n">
-        <v>0</v>
+      <c r="N34" s="6" t="n"/>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6" t="n"/>
+      <c r="Q34" s="6" t="inlineStr">
+        <is>
+          <t>The last election: the game ends after this turn. Worth 1 prestige for each election card you hold, this one included.</t>
+        </is>
+      </c>
+      <c r="R34" s="6" t="inlineStr">
+        <is>
+          <t>Secession</t>
+        </is>
+      </c>
+      <c r="S34" s="6" t="inlineStr">
+        <is>
+          <t>Each paper destroys the cheapest card in its hand.</t>
+        </is>
+      </c>
+      <c r="T34" s="5" t="inlineStr">
+        <is>
+          <t>destroy_cheapest</t>
+        </is>
       </c>
       <c r="U34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V34" s="5" t="n"/>
-      <c r="W34" s="6" t="inlineStr">
-        <is>
-          <t>The last election: the game ends after this turn. Worth 1 prestige for each election card you hold, this one included.</t>
-        </is>
-      </c>
-      <c r="X34" s="6" t="inlineStr">
-        <is>
-          <t>Secession</t>
-        </is>
-      </c>
-      <c r="Y34" s="6" t="inlineStr">
-        <is>
-          <t>Each paper destroys the cheapest card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z34" s="5" t="inlineStr">
-        <is>
-          <t>destroy_cheapest</t>
-        </is>
-      </c>
-      <c r="AA34" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -15165,57 +14531,35 @@
       <c r="M35" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="N35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" s="5" t="n">
-        <v>0</v>
+      <c r="N35" s="6" t="n"/>
+      <c r="O35" s="6" t="n"/>
+      <c r="P35" s="6" t="n"/>
+      <c r="Q35" s="6" t="inlineStr">
+        <is>
+          <t>The last election: the game ends after this turn. Worth 2 prestige, plus 1 for each election card you hold, this one included.</t>
+        </is>
+      </c>
+      <c r="R35" s="6" t="inlineStr">
+        <is>
+          <t>Secession</t>
+        </is>
+      </c>
+      <c r="S35" s="6" t="inlineStr">
+        <is>
+          <t>Each paper destroys the cheapest card in its hand.</t>
+        </is>
+      </c>
+      <c r="T35" s="5" t="inlineStr">
+        <is>
+          <t>destroy_cheapest</t>
+        </is>
       </c>
       <c r="U35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" s="5" t="n"/>
-      <c r="W35" s="6" t="inlineStr">
-        <is>
-          <t>The last election: the game ends after this turn. Worth 2 prestige, plus 1 for each election card you hold, this one included.</t>
-        </is>
-      </c>
-      <c r="X35" s="6" t="inlineStr">
-        <is>
-          <t>Secession</t>
-        </is>
-      </c>
-      <c r="Y35" s="6" t="inlineStr">
-        <is>
-          <t>Each paper destroys the cheapest card in its hand.</t>
-        </is>
-      </c>
-      <c r="Z35" s="5" t="inlineStr">
-        <is>
-          <t>destroy_cheapest</t>
-        </is>
-      </c>
-      <c r="AA35" s="5" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA35"/>
+  <autoFilter ref="A1:U35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>